<commit_message>
Add gas installation calculations and reference drawings
</commit_message>
<xml_diff>
--- a/00_Data/Datos curso 2026.xlsx
+++ b/00_Data/Datos curso 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\00_MiTrabajo\Asig__ INSTALACIONES 2 Grado Mecanica\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Unidades compartidas\Practicas_Inst2\5_Gas_natural\00_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8088345F-3FC0-476B-B7D2-8FD45799513E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91BEDFCA-0B46-45B1-9468-F8DC0F5CC20D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -461,10 +461,10 @@
     <t>Horno kW</t>
   </si>
   <si>
-    <t>PCS (kWh/m3(s))</t>
-  </si>
-  <si>
     <t>PCS (MJ/m3(s))</t>
+  </si>
+  <si>
+    <t>Secadora(KW)</t>
   </si>
 </sst>
 </file>
@@ -500,6 +500,7 @@
     <font>
       <sz val="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -909,28 +910,28 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N46"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" style="3"/>
-    <col min="2" max="2" width="19.125" customWidth="1"/>
-    <col min="3" max="3" width="18.125" customWidth="1"/>
-    <col min="4" max="4" width="15.125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="19.09765625" customWidth="1"/>
+    <col min="3" max="3" width="18.09765625" customWidth="1"/>
+    <col min="4" max="4" width="15.09765625" style="3" customWidth="1"/>
     <col min="5" max="5" width="13" style="3" customWidth="1"/>
-    <col min="6" max="7" width="14.125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="13.375" style="3" customWidth="1"/>
+    <col min="6" max="7" width="14.09765625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="13.3984375" style="3" customWidth="1"/>
     <col min="9" max="10" width="11" style="3"/>
-    <col min="11" max="11" width="13.625" style="3" customWidth="1"/>
-    <col min="12" max="12" width="12.875" style="3" customWidth="1"/>
+    <col min="11" max="11" width="13.59765625" style="3" customWidth="1"/>
+    <col min="12" max="12" width="12.8984375" style="3" customWidth="1"/>
     <col min="13" max="13" width="11" style="3"/>
-    <col min="14" max="14" width="37.625" customWidth="1"/>
+    <col min="14" max="14" width="37.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="18" x14ac:dyDescent="0.35">
       <c r="B1" s="4" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>122</v>
       </c>
@@ -962,17 +963,17 @@
         <v>140</v>
       </c>
       <c r="K3" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>142</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>16</v>
       </c>
@@ -1011,7 +1012,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>17</v>
       </c>
@@ -1034,7 +1035,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>25</v>
       </c>
@@ -1057,7 +1058,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>27</v>
       </c>
@@ -1080,7 +1081,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>1</v>
       </c>
@@ -1119,7 +1120,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>2</v>
       </c>
@@ -1142,7 +1143,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>3</v>
       </c>
@@ -1165,7 +1166,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>4</v>
       </c>
@@ -1188,7 +1189,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>5</v>
       </c>
@@ -1227,7 +1228,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>6</v>
       </c>
@@ -1250,7 +1251,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>7</v>
       </c>
@@ -1273,7 +1274,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>8</v>
       </c>
@@ -1296,7 +1297,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>10</v>
       </c>
@@ -1335,7 +1336,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>11</v>
       </c>
@@ -1358,7 +1359,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>12</v>
       </c>
@@ -1381,7 +1382,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>123</v>
       </c>
@@ -1398,7 +1399,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>42</v>
       </c>
@@ -1421,7 +1422,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>14</v>
       </c>
@@ -1460,7 +1461,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>18</v>
       </c>
@@ -1483,7 +1484,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>19</v>
       </c>
@@ -1506,7 +1507,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>20</v>
       </c>
@@ -1529,7 +1530,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>21</v>
       </c>
@@ -1568,7 +1569,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>23</v>
       </c>
@@ -1591,7 +1592,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>28</v>
       </c>
@@ -1614,7 +1615,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>29</v>
       </c>
@@ -1637,7 +1638,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>32</v>
       </c>
@@ -1676,7 +1677,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>33</v>
       </c>
@@ -1699,7 +1700,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="31" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>34</v>
       </c>
@@ -1729,7 +1730,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>79</v>
       </c>
@@ -1746,7 +1747,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
         <v>35</v>
       </c>
@@ -1785,7 +1786,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="3">
         <v>36</v>
       </c>
@@ -1808,7 +1809,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="3">
         <v>37</v>
       </c>
@@ -1831,7 +1832,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>38</v>
       </c>
@@ -1854,7 +1855,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>39</v>
       </c>
@@ -1893,7 +1894,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
         <v>40</v>
       </c>
@@ -1916,7 +1917,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>41</v>
       </c>
@@ -1939,7 +1940,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>126</v>
       </c>
@@ -1956,7 +1957,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="3">
         <v>13</v>
       </c>
@@ -1971,7 +1972,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="3">
         <v>15</v>
       </c>
@@ -1988,7 +1989,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" s="3">
         <v>22</v>
       </c>
@@ -2005,7 +2006,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" s="3">
         <v>24</v>
       </c>
@@ -2023,7 +2024,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="3">
         <v>26</v>
       </c>
@@ -2040,7 +2041,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" s="3">
         <v>31</v>
       </c>

</xml_diff>